<commit_message>
Corrida | GR-EPRIV-INF | 2026-06-17 11:34:11.685179
</commit_message>
<xml_diff>
--- a/indicadores/GR-EPRIV-INF_out.xlsx
+++ b/indicadores/GR-EPRIV-INF_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Ocupados informales en el sector privado del Gran Rosario</t>
+    <t xml:space="preserve">Ocupados informales en el sector privado</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aglomerado Gran Rosario</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">vcorvalan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1086,9 +1092,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1099,7 +1109,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1113,12 +1123,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>-0.234116698817283</v>
+        <v>-0.227429780760657</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1129,7 +1139,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1157,7 +1167,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1171,12 +1181,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0395045978888794</v>
+        <v>0.038995877860649</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1199,7 +1209,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1213,7 +1223,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1227,7 +1237,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1241,12 +1251,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.661942796338858</v>
+        <v>0.673305892777082</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1257,7 +1267,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1271,12 +1281,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.455952867215112</v>
+        <v>0.514476773648625</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1419,10 +1429,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1435,10 +1445,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1462,66 +1472,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>184.844</v>
@@ -1574,7 +1584,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>187.087</v>
@@ -1631,7 +1641,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>186.517</v>
@@ -1688,7 +1698,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>189.606</v>
@@ -1745,7 +1755,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>178.421</v>
@@ -1804,7 +1814,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>183.734</v>
@@ -1863,7 +1873,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>190.427</v>
@@ -1922,7 +1932,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>190.167</v>
@@ -1981,7 +1991,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>186.12</v>
@@ -2040,7 +2050,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>178.072</v>
@@ -2099,7 +2109,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>188.752</v>
@@ -2158,7 +2168,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>185.205</v>
@@ -2217,7 +2227,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>175.164</v>
@@ -2276,7 +2286,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>163.593</v>
@@ -2335,7 +2345,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>188.0315</v>
@@ -2394,7 +2404,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>191.384</v>
@@ -2453,7 +2463,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>174.593</v>
@@ -2512,7 +2522,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>179.795</v>
@@ -2571,7 +2581,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>187.311</v>
@@ -2630,7 +2640,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>184.615</v>
@@ -2689,7 +2699,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>194.435</v>
@@ -2748,7 +2758,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>169.467</v>
@@ -2807,7 +2817,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>178.154</v>
@@ -2866,7 +2876,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>186.889</v>
@@ -2925,7 +2935,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>195.657</v>
@@ -2984,7 +2994,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>183.563</v>
@@ -3043,7 +3053,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>173.725</v>
@@ -3102,7 +3112,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>176.801</v>
@@ -3161,7 +3171,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>171.71</v>
@@ -3220,7 +3230,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>181.36</v>
@@ -3279,7 +3289,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>181.025</v>
@@ -3338,7 +3348,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>176.741</v>
@@ -3397,7 +3407,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>168.454</v>
@@ -3456,7 +3466,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>182.36</v>
@@ -3515,7 +3525,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>171.866</v>
@@ -3574,7 +3584,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>160.682</v>
@@ -3633,7 +3643,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>166.629</v>
@@ -3692,7 +3702,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>186.602</v>
@@ -3751,7 +3761,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>197.311</v>
@@ -3810,7 +3820,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>188.755</v>
@@ -3869,7 +3879,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>184.912</v>
@@ -3928,7 +3938,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>173.805</v>
@@ -3987,7 +3997,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>193.59</v>
@@ -4046,7 +4056,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>209.016</v>
@@ -4105,7 +4115,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>196.596</v>
@@ -4164,7 +4174,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>198.82</v>
@@ -4223,7 +4233,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>188.675</v>
@@ -4282,7 +4292,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>187.299</v>
@@ -4341,7 +4351,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>183.9625</v>
@@ -4400,7 +4410,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>186.559</v>
@@ -4459,7 +4469,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>183.76</v>
@@ -4518,7 +4528,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>165.582</v>
@@ -4577,7 +4587,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>171.329</v>
@@ -4636,7 +4646,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>196.137</v>
@@ -4695,7 +4705,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>171.817</v>
@@ -4754,7 +4764,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>159.256</v>
@@ -4813,7 +4823,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>189.021</v>
@@ -4872,7 +4882,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>203.006</v>
@@ -4931,7 +4941,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>181.525</v>
@@ -4990,7 +5000,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>174.433</v>
@@ -5049,7 +5059,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>192.638</v>
@@ -5108,7 +5118,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>192.737</v>
@@ -5167,7 +5177,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>178.853</v>
@@ -5226,7 +5236,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>191.494</v>
@@ -5285,7 +5295,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>202.1</v>
@@ -5344,7 +5354,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>137.864</v>
@@ -5403,7 +5413,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>163.457</v>
@@ -5462,7 +5472,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>180.02</v>
@@ -5521,7 +5531,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>206.268</v>
@@ -5580,7 +5590,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>188.803</v>
@@ -5639,7 +5649,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>205.667</v>
@@ -5698,7 +5708,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>185.9</v>
@@ -5757,7 +5767,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>205.218</v>
@@ -5816,7 +5826,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>213.262</v>
@@ -5875,7 +5885,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>215.168</v>
@@ -5934,7 +5944,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>223.64</v>
@@ -5993,7 +6003,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>226.867</v>
@@ -6052,7 +6062,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>220.115</v>
@@ -6111,7 +6121,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>200.998</v>
@@ -6170,7 +6180,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>193.143</v>
@@ -6229,7 +6239,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>210.215</v>
@@ -6288,7 +6298,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>233.918</v>
@@ -6347,7 +6357,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>217.826</v>
@@ -6406,7 +6416,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>201.979</v>
@@ -6465,7 +6475,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>218.523</v>
@@ -6524,7 +6534,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>259.799</v>
@@ -6583,7 +6593,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>223.724</v>
@@ -6642,7 +6652,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>223.584</v>
@@ -6701,7 +6711,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2"/>
       <c r="C90" s="3" t="n">
@@ -6734,7 +6744,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2"/>
       <c r="C91" s="3" t="n">
@@ -6767,7 +6777,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2"/>
       <c r="C92" s="3" t="n">
@@ -6800,7 +6810,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2"/>
       <c r="C93" s="3" t="n">
@@ -6833,7 +6843,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2"/>
       <c r="C94" s="3"/>
@@ -6856,7 +6866,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2"/>
       <c r="C95" s="3"/>
@@ -6879,7 +6889,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
@@ -6902,7 +6912,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="3"/>
@@ -6925,7 +6935,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2"/>
       <c r="C98" s="3"/>
@@ -6948,7 +6958,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2"/>
       <c r="C99" s="3"/>
@@ -6971,7 +6981,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2"/>
       <c r="C100" s="3"/>
@@ -6994,7 +7004,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2"/>
       <c r="C101" s="3"/>
@@ -7017,7 +7027,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2"/>
       <c r="C102" s="3"/>
@@ -7040,7 +7050,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2"/>
       <c r="C103" s="3"/>
@@ -7063,7 +7073,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2"/>
       <c r="C104" s="3"/>
@@ -7086,7 +7096,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2"/>
       <c r="C105" s="3"/>
@@ -7109,7 +7119,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2"/>
       <c r="C106" s="3"/>
@@ -7132,7 +7142,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2"/>
       <c r="C107" s="3"/>
@@ -7155,7 +7165,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2"/>
       <c r="C108" s="3"/>
@@ -7178,7 +7188,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2"/>
       <c r="C109" s="3"/>
@@ -7212,97 +7222,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -7326,7 +7336,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -7336,80 +7346,80 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.173164063293851</v>
+        <v>-0.168159348791623</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.138709406221347</v>
+        <v>-0.136509896938198</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.108842455893944</v>
+        <v>-0.11340327541941</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0391864012261878</v>
+        <v>0.0301876153557199</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.198757636051749</v>
+        <v>0.19747373967353</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.212661182770697</v>
+        <v>0.218167362850277</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.0763193656971647</v>
+        <v>0.0778593441887351</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.130224129393615</v>
+        <v>-0.128855970090904</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.234116698817283</v>
+        <v>-0.227429780760657</v>
       </c>
     </row>
     <row r="14">

</xml_diff>